<commit_message>
Tracker: add Google Maps, uniforms and Notion knowledge base tasks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D49MhKTUUBcnS2eWubqeXM
</commit_message>
<xml_diff>
--- a/AURA_task_tracker.xlsx
+++ b/AURA_task_tracker.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Сводка" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Задачи'!$A$4:$M$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Задачи'!$A$4:$M$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M23"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -549,7 +549,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Создан 26.10.2026 по итогам созвона. Обновлять статусы еженедельно.</t>
+          <t>Создан 26.10.2026 по итогам созвона, обновлён 30.10.2026. Обновлять статусы еженедельно.</t>
         </is>
       </c>
     </row>
@@ -742,15 +742,133 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
+          <t>Организационное</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Создать базу знаний в Notion</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>• Структура: компания и команда, услуги и прайс, Hemaya и лицензии, сегменты и конкуренты, маркетинг и контент, продажи (воронка, скрипты, шаблоны КП), онбординг новых сотрудников
+• Перенести готовые материалы (выжимки по конкурентам, сегментам, Hemaya, LinkedIn, SEO-аудит, сравнение CRM)
+• Выдать доступы команде, договориться, кто что обновляет</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>База знаний в Notion, команда пользуется; новый сейл и инженер онбордятся по ней</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Маркетолог (я)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Анастасия (рабочий аккаунт), вся команда — доступ</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>46339</v>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="L7" s="7">
+        <f>IF(K7="Готово","",J7-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M7" s="8" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Организационное</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Спецодежда для инженеров и монтажников</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>• Уточнить объём задачи: для кого (инженер с 9.11, монтажники), сколько комплектов и что входит (футболки/поло, брюки, кепки, жилеты)
+• Требования: лёгкая ткань под жару, светоотражающие элементы для объектов, логотип AURA и контакты
+• Макет брендирования
+• Запросить 2–3 предложения у поставщиков в ОАЭ (цена, сроки)
+• Согласовать и заказать</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Спецодежда заказана, к выходу монтажников команда в брендированной форме</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Маркетолог (я)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Антон (бюджет, согласование), Игнат (кол-во и размеры)</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Средний</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>46335</v>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="L8" s="7">
+        <f>IF(K8="Готово","",J8-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
           <t>Доступы</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Доступ к сайту</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>• Админка / CMS или репозиторий сайта (Next.js)
 • Хостинг и домен — кто владелец
@@ -758,316 +876,202 @@
 • Кто вносит правки: я или Роман</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Есть рабочие доступы, понятен порядок внесения правок</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Анастасия, Роман</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n">
+      <c r="I9" s="6" t="n">
         <v>46321</v>
       </c>
-      <c r="J7" s="6" t="n">
+      <c r="J9" s="6" t="n">
         <v>46323</v>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L7" s="7">
-        <f>IF(K7="Готово","",J7-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M7" s="8" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="L9" s="7">
+        <f>IF(K9="Готово","",J9-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Доступы</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Рабочий Google-аккаунт</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>• Получить рабочий аккаунт (почта на домене или общий)
 • Доступ к общему Google Drive с материалами
 • Подключить к GA4, Search Console, будущему Google Business Profile</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E10" s="5" t="inlineStr">
         <is>
           <t>Работаю из рабочего аккаунта, все материалы в общей папке</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>Анастасия / Антон</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I8" s="6" t="n">
+      <c r="I10" s="6" t="n">
         <v>46321</v>
       </c>
-      <c r="J8" s="6" t="n">
+      <c r="J10" s="6" t="n">
         <v>46323</v>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L8" s="7">
-        <f>IF(K8="Готово","",J8-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M8" s="8" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="L10" s="7">
+        <f>IF(K10="Готово","",J10-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Доступы</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Доступ к Facebook-странице и LinkedIn</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>• Роль администратора/редактора страницы Facebook
 • Доступ к Meta Business Suite
 • Доступ к странице компании в LinkedIn (если есть) и к профилю Антона для публикаций — по согласованию</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Могу публиковать и смотреть статистику в FB и LinkedIn</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Анастасия, Антон, Роман</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I9" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>46321</v>
       </c>
-      <c r="J9" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>46324</v>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L9" s="7">
-        <f>IF(K9="Готово","",J9-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M9" s="8" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="L11" s="7">
+        <f>IF(K11="Готово","",J11-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Контент</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Получить актуальный контент-план</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>• Забрать у Романа текущий контент-план и статус постов (что опубликовано, что в работе)
 • Свести с имеющимися материалами: 8 готовых постов RU/EN, 30 идей, сценарии видео Антона
 • Определить каналы и частоту</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Единый контент-план с датами публикаций на ноябрь</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G12" s="5" t="inlineStr">
         <is>
           <t>Роман, Анастасия</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I10" s="6" t="n">
+      <c r="I12" s="6" t="n">
         <v>46321</v>
-      </c>
-      <c r="J10" s="6" t="n">
-        <v>46325</v>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Не начато</t>
-        </is>
-      </c>
-      <c r="L10" s="7">
-        <f>IF(K10="Готово","",J10-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M10" s="8" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Презентации</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Собрать текущие презентации и материалы</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>• Получить от Романа все презентации, листовки, sales kit с пакетами цен
-• Зафиксировать, какие презентации в работе и для кого</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Все материалы в общей папке, понятен статус каждой презентации</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>Маркетолог (я)</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>Роман, Анастасия</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>Высокий</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="n">
-        <v>46321</v>
-      </c>
-      <c r="J11" s="6" t="n">
-        <v>46323</v>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Не начато</t>
-        </is>
-      </c>
-      <c r="L11" s="7">
-        <f>IF(K11="Готово","",J11-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M11" s="8" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Презентации</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Определить список презентаций и ТЗ к ним</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>• Согласовать с Антоном, какие презентации нужны в первую очередь (напр. общая B2B, B2C для вилл, AMC/сервис)
-• Для каждой: аудитория, цель, структура, что показываем (лицензии, процесс, оборудование, цены)</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Утверждённый список презентаций с ТЗ и приоритетом</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Маркетолог (я)</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Антон</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Высокий</t>
-        </is>
-      </c>
-      <c r="I12" s="6" t="n">
-        <v>46323</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>46325</v>
@@ -1094,124 +1098,238 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
+          <t>Собрать текущие презентации и материалы</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>• Получить от Романа все презентации, листовки, sales kit с пакетами цен
+• Зафиксировать, какие презентации в работе и для кого</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Все материалы в общей папке, понятен статус каждой презентации</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Маркетолог (я)</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>Роман, Анастасия</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Высокий</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>46321</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="L13" s="7">
+        <f>IF(K13="Готово","",J13-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Презентации</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Определить список презентаций и ТЗ к ним</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>• Согласовать с Антоном, какие презентации нужны в первую очередь (напр. общая B2B, B2C для вилл, AMC/сервис)
+• Для каждой: аудитория, цель, структура, что показываем (лицензии, процесс, оборудование, цены)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Утверждённый список презентаций с ТЗ и приоритетом</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Маркетолог (я)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Антон</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Высокий</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>46323</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="L14" s="7">
+        <f>IF(K14="Готово","",J14-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Презентации</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
           <t>Подготовить презентацию №1 (приоритетная)</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>• Структура и тексты (EN, при необходимости RU)
 • Дизайн в стиле сайта/бренда
 • Согласование с Антоном, правки</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr">
         <is>
           <t>Финальная версия PDF + редактируемый исходник</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>Антон (согласование), Роман (дизайн — при необходимости)</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I13" s="6" t="n">
+      <c r="I15" s="6" t="n">
         <v>46325</v>
       </c>
-      <c r="J13" s="6" t="n">
+      <c r="J15" s="6" t="n">
         <v>46331</v>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L13" s="7">
-        <f>IF(K13="Готово","",J13-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M13" s="8" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="L15" s="7">
+        <f>IF(K15="Готово","",J15-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>Презентации</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Подготовить презентацию №2</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>• По тому же процессу, что №1</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Финальная версия PDF + исходник</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>Антон</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>Средний</t>
         </is>
       </c>
-      <c r="I14" s="6" t="n">
+      <c r="I16" s="6" t="n">
         <v>46331</v>
       </c>
-      <c r="J14" s="6" t="n">
+      <c r="J16" s="6" t="n">
         <v>46338</v>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L14" s="7">
-        <f>IF(K14="Готово","",J14-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M14" s="8" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="L16" s="7">
+        <f>IF(K16="Готово","",J16-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>CRM</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Сформулировать требования к CRM</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>• Простая, недорогая, с мобильным приложением
 • Интеграция с WhatsApp (основной канал заявок) и формой сайта
@@ -1219,173 +1337,173 @@
 • Кто пользуется: Антон, сейл, Игнат/инженер</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E17" s="5" t="inlineStr">
         <is>
           <t>Список требований, согласованный с Антоном</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>Антон, Анастасия</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I15" s="6" t="n">
+      <c r="I17" s="6" t="n">
         <v>46322</v>
       </c>
-      <c r="J15" s="6" t="n">
+      <c r="J17" s="6" t="n">
         <v>46325</v>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L15" s="7">
-        <f>IF(K15="Готово","",J15-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M15" s="8" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="L17" s="7">
+        <f>IF(K17="Готово","",J17-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>CRM</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Сравнить варианты и выбрать CRM</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>• Сравнить 3–4 простые CRM (напр. Kommo, Bitrix24, Pipedrive, Zoho Bigin, HubSpot Free): цена, WhatsApp, удобство
 • Короткая таблица сравнения + рекомендация</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Выбрана CRM, понятна стоимость</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>Антон (решение)</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I16" s="6" t="n">
+      <c r="I18" s="6" t="n">
         <v>46325</v>
       </c>
-      <c r="J16" s="6" t="n">
+      <c r="J18" s="6" t="n">
         <v>46330</v>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K18" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L16" s="7">
-        <f>IF(K16="Готово","",J16-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M16" s="8" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="L18" s="7">
+        <f>IF(K18="Готово","",J18-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>CRM</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Настроить CRM</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>• Завести воронки (из задачи «Воронка»), поля, источники лидов
 • Подключить WhatsApp и форму сайта
 • Короткая инструкция для команды</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>CRM работает, тестовый лид проходит путь от заявки до сделки</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>Антон</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I17" s="6" t="n">
+      <c r="I19" s="6" t="n">
         <v>46335</v>
       </c>
-      <c r="J17" s="6" t="n">
+      <c r="J19" s="6" t="n">
         <v>46339</v>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K19" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L17" s="7">
-        <f>IF(K17="Готово","",J17-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M17" s="8" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="L19" s="7">
+        <f>IF(K19="Готово","",J19-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Продажи</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Описать воронку для мелких B2B и B2C</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>• Этапы: заявка → квалификация → аудит/выезд → КП → сделка → монтаж → сервис/AMC
 • Критерии квалификации лида и порог, после которого сделку ведёт Антон
@@ -1393,58 +1511,58 @@
 • Отдельно для B2C (виллы) и малого B2B</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
+      <c r="E20" s="5" t="inlineStr">
         <is>
           <t>Документ с воронкой, согласованный с Антоном и Игнатом; основа для настройки CRM</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>Антон, Игнат</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I18" s="6" t="n">
+      <c r="I20" s="6" t="n">
         <v>46324</v>
       </c>
-      <c r="J18" s="6" t="n">
+      <c r="J20" s="6" t="n">
         <v>46332</v>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="K20" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L18" s="7">
-        <f>IF(K18="Готово","",J18-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M18" s="8" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="L20" s="7">
+        <f>IF(K20="Готово","",J20-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>Продажи</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Прописать критерии поиска сейла</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>• Профиль: опыт продаж в ОАЭ (security/ELV/стройка), языки EN (+AR/RU плюс)
 • Обязанности: входящие лиды, мелкие B2B и B2C, ведение CRM
@@ -1452,58 +1570,58 @@
 • Где искать: LinkedIn, Bayt, Dubizzle, рекомендации</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
         <is>
           <t>Портрет кандидата + текст вакансии, согласованные с Антоном</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>Антон, Анастасия</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I19" s="6" t="n">
+      <c r="I21" s="6" t="n">
         <v>46322</v>
       </c>
-      <c r="J19" s="6" t="n">
+      <c r="J21" s="6" t="n">
         <v>46326</v>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L19" s="7">
-        <f>IF(K19="Готово","",J19-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M19" s="8" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="L21" s="7">
+        <f>IF(K21="Готово","",J21-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Стратегия LinkedIn</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>• Что ведём: страница компании и/или личный профиль Антона
 • Аудит профиля Антона, правки шапки и описания
@@ -1512,222 +1630,281 @@
 • Метрики</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>Документ стратегии + контент-план LinkedIn на ноябрь</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>Антон</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I20" s="6" t="n">
+      <c r="I22" s="6" t="n">
         <v>46325</v>
       </c>
-      <c r="J20" s="6" t="n">
+      <c r="J22" s="6" t="n">
         <v>46333</v>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="K22" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L20" s="7">
-        <f>IF(K20="Готово","",J20-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M20" s="8" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="L22" s="7">
+        <f>IF(K22="Готово","",J22-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Настроить кросспостинг LinkedIn → Facebook</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>• Выбрать способ (Meta Business Suite / Buffer или аналог / вручную)
 • Адаптировать формат постов под FB
 • Проверить на 2–3 публикациях</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Посты из LinkedIn регулярно выходят в Facebook</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Доступы к FB и LinkedIn</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>Средний</t>
         </is>
       </c>
-      <c r="I21" s="6" t="n">
+      <c r="I23" s="6" t="n">
         <v>46333</v>
       </c>
-      <c r="J21" s="6" t="n">
+      <c r="J23" s="6" t="n">
         <v>46337</v>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L21" s="7">
-        <f>IF(K21="Готово","",J21-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M21" s="8" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="L23" s="7">
+        <f>IF(K23="Готово","",J23-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>Лидогенерация</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Добавить организацию в Google Maps (Google Business Profile)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>• Создать профиль с рабочего Google-аккаунта: название «AURA Reinvent Security Systems», категории (CCTV / security system installer), адрес RAKEZ Compass Building, Al Hamra Industrial Zone-FZ, телефон/WhatsApp, сайт, часы работы, зона обслуживания (RAK и Северные эмираты)
+• Пройти верификацию Google (видео / открытка — сроки зависят от Google)
+• Добавить услуги, описание, фото (команда, объекты, логотип)
+• Ссылку на профиль — на сайт и в соцсети
+• Запустить сбор отзывов после каждого объекта</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Профиль подтверждён и виден в Google Maps по запросам «CCTV Ras Al Khaimah», появились первые отзывы</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Маркетолог (я)</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Рабочий Google-аккаунт, Антон (адрес, часы, фото)</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Высокий</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>46325</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>46333</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Не начато</t>
+        </is>
+      </c>
+      <c r="L24" s="7">
+        <f>IF(K24="Готово","",J24-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Лидогенерация</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Подготовка к лидогенерации</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>• Google Business Profile (Google Maps) — создать/проверить, сбор отзывов
-• Цели в GA4: клики в WhatsApp, отправка формы
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>• Цели в GA4: клики в WhatsApp, отправка формы
 • UTM-метки для всех каналов
 • Посадочная под бесплатный аудит — проверить и улучшить
 • База ЛПР приоритетных сегментов для аутрича
 • Лицензии на сайт (страница /licenses) — запросить у Антона</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t>Каналы готовы к запуску, заявки отслеживаются и попадают в CRM</t>
         </is>
       </c>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>Антон, доступ к сайту и Google</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I22" s="6" t="n">
+      <c r="I25" s="6" t="n">
         <v>46335</v>
       </c>
-      <c r="J22" s="6" t="n">
+      <c r="J25" s="6" t="n">
         <v>46346</v>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L22" s="7">
-        <f>IF(K22="Готово","",J22-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M22" s="8" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="L25" s="7">
+        <f>IF(K25="Готово","",J25-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Лидогенерация</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Запуск лидогенерации</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>• Старт публикаций и аутрича по плану
 • Еженедельный отчёт: лиды, источники, конверсия</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>Первые лиды в CRM, еженедельный отчёт</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Маркетолог (я)</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>Сейл (если нанят), Антон</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>Высокий</t>
         </is>
       </c>
-      <c r="I23" s="6" t="n">
+      <c r="I26" s="6" t="n">
         <v>46342</v>
       </c>
-      <c r="J23" s="6" t="n">
+      <c r="J26" s="6" t="n">
         <v>46356</v>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Не начато</t>
         </is>
       </c>
-      <c r="L23" s="7">
-        <f>IF(K23="Готово","",J23-TODAY())</f>
-        <v/>
-      </c>
-      <c r="M23" s="8" t="n"/>
+      <c r="L26" s="7">
+        <f>IF(K26="Готово","",J26-TODAY())</f>
+        <v/>
+      </c>
+      <c r="M26" s="8" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M23"/>
-  <conditionalFormatting sqref="A5:M23">
+  <autoFilter ref="A4:M26"/>
+  <conditionalFormatting sqref="A5:M26">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$K5="Готово"</formula>
     </cfRule>
@@ -1735,7 +1912,7 @@
       <formula>AND($K5&lt;&gt;"Готово",$K5&lt;&gt;"Отменено",$J5&lt;TODAY())</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K23">
+  <conditionalFormatting sqref="K5:K26">
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"В работе"</formula>
     </cfRule>
@@ -1743,16 +1920,16 @@
       <formula>"Ждёт доступа"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H23">
+  <conditionalFormatting sqref="H5:H26">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"Высокий"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="K5:K23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K5:K26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Не начато,В работе,На согласовании,Ждёт доступа,Готово,Отменено"</formula1>
     </dataValidation>
-    <dataValidation sqref="H5:H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Высокий,Средний,Низкий"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1766,7 +1943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1799,7 +1976,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A4)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A4)</f>
         <v/>
       </c>
     </row>
@@ -1810,7 +1987,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A5)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A5)</f>
         <v/>
       </c>
     </row>
@@ -1821,7 +1998,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A6)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A6)</f>
         <v/>
       </c>
     </row>
@@ -1832,7 +2009,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A7)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A7)</f>
         <v/>
       </c>
     </row>
@@ -1843,7 +2020,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A8)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A8)</f>
         <v/>
       </c>
     </row>
@@ -1854,7 +2031,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF(Задачи!$K$5:$K$23,A9)</f>
+        <f>COUNTIF(Задачи!$K$5:$K$26,A9)</f>
         <v/>
       </c>
     </row>
@@ -1865,7 +2042,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTA(Задачи!$C$5:$C$23)</f>
+        <f>COUNTA(Задачи!$C$5:$C$26)</f>
         <v/>
       </c>
     </row>
@@ -1876,7 +2053,7 @@
         </is>
       </c>
       <c r="B11">
-        <f>COUNTIFS(Задачи!$J$5:$J$23,"&lt;"&amp;TODAY(),Задачи!$K$5:$K$23,"&lt;&gt;Готово",Задачи!$K$5:$K$23,"&lt;&gt;Отменено")</f>
+        <f>COUNTIFS(Задачи!$J$5:$J$26,"&lt;"&amp;TODAY(),Задачи!$K$5:$K$26,"&lt;&gt;Готово",Задачи!$K$5:$K$26,"&lt;&gt;Отменено")</f>
         <v/>
       </c>
     </row>
@@ -1938,22 +2115,46 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>13.11</t>
+          <t>07.11</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CRM настроена</t>
+          <t>Профиль в Google Maps создан и отправлен на верификацию</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>09.11</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Спецодежда заказана</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>13.11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>CRM настроена, база знаний в Notion готова</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>16–30.11</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Запуск лидогенерации</t>
         </is>

</xml_diff>